<commit_message>
Leads: 2026-09-28 00:06 UTC (cycle 148)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,62 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Comfort Caddies Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>comfortcaddies.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://comfortcaddies.com/services/heat-pumps/heat-pump-installation/</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>website@comfortcaddies.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>239-426-8581</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Naples FL</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>heat pump installation Naples FL</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 05:44 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -584,7 +584,6 @@
           <t>https://comfortcaddies.com/services/heat-pumps/heat-pump-installation/</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>website@comfortcaddies.com</t>
@@ -614,6 +613,66 @@
         </is>
       </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Rick The Plumber | Serving Peoria, AZ, Arizona</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ricktheplumberaz.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://ricktheplumberaz.com/peoria-az</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>For Peoria</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>info@ricktheplumberaz.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(602) 481-8428</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Peoria AZ</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>90</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>plumber Peoria AZ</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 05:47 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -678,6 +678,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Oh My Roof Construction &amp; Roofing</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ohmyroofconstruction.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://ohmyroofconstruction.com/our-services/roof-replacement-lafayette-la/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Work That</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>info@ohmyroofconstruction.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(337) 233-2571</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Lafayette LA</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>100</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>roof replacement Lafayette LA</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 05:50 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -738,6 +738,66 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>123 Remodeling &amp; Roofing</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>123remodelingok.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.123remodelingok.com/service-area/edmond</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Partner Kris</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>help@123remodelingok.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(405) 208-4006</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Edmond OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>roof replacement Edmond OK</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 05:51 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -798,6 +798,66 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Colorado Preferred Roofing</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>coloradopreferredroofing.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://coloradopreferredroofing.com/service-areas/lakewood/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>What Makes</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>info@coloradopreferredroofing.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(303) 766-3102</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Lakewood CO</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>roofing contractor Lakewood CO</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 05:53 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -858,6 +858,182 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>All Clear Pumping &amp; Sewer</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>allclearmo.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://www.allclearmo.com/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Owners Shawn</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>contact@allclearmo.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>573-634-0165</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Columbia MO</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>94</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>sewer repair Columbia MO</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Michels Plumbing, Inc.</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>michelsplumbing.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://www.michelsplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>info@michelsplumbing.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(630) 801-9700</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Aurora IL</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>78</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>plumbing company Aurora IL</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>West Palm Beach Roofing Contractors: 20 Compared (2026)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>floridaroofingdirectory.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://floridaroofingdirectory.com/blog/best-roofing-companies-west-palm-beach-florida</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>By Shelly</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>hal@floridaroofingdirectory.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>561-872-3630</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>West Palm Beach FL</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>76</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>roofing contractor West Palm Beach FL</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 05:54 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -939,7 +939,6 @@
           <t>https://www.michelsplumbing.com/</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>info@michelsplumbing.com</t>
@@ -1029,6 +1028,66 @@
         </is>
       </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Comfortable Air Services</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>comfortableairservices.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.comfortableairservices.com/areas-we-serve/arlington-va/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Email Us</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>johnsmith@gmail.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(703) 590-7517</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Arlington VA</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>90</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>water heater repair Arlington VA</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 05:56 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1093,6 +1093,122 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Hanes Mechanical, Inc.</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>hanesmechanical.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.hanesmechanical.com/york/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>info@hanesmechanical.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(717) 832-9004</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>York PA</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>100</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>HVAC contractor York PA</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PORTILLO CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>portilloroofs.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://portilloroofs.com/roof-replacement-peoria-il/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Portillo Construction</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>info@portilloroofs.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(309) 328-7663</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Peoria IL</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>roof replacement Peoria IL</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 06:03 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1114,7 +1114,6 @@
           <t>https://www.hanesmechanical.com/york/</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>info@hanesmechanical.com</t>
@@ -1204,6 +1203,58 @@
         </is>
       </c>
       <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Orlando Roofing</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>orlando-roofing.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://orlando-roofing.com/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>info@orlando-roofing.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Orlando FL</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>86</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>roofing contractor Orlando FL</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 06:09 UTC (cycle 19)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1229,13 +1229,11 @@
           <t>https://orlando-roofing.com/</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>info@orlando-roofing.com</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>Orlando FL</t>
@@ -1255,6 +1253,62 @@
         </is>
       </c>
       <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>HeatCoolVT-Homepage</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>heatcoolvt.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.heatcoolvt.com/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>contact@heatcoolvt.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>802.658.3286</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Burlington VT</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>64</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>heating and cooling company Burlington VT</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 06:21 UTC (cycle 27)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1279,7 +1279,6 @@
           <t>https://www.heatcoolvt.com/</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>contact@heatcoolvt.com</t>
@@ -1309,6 +1308,66 @@
         </is>
       </c>
       <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>www.karmabuilders.org</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>karmabuilders.org</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://www.karmabuilders.org/roofing-company-cranston-ri</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Roofing Company</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>karmabuildersma@gmail.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>508-965-8538</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Cranston RI</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>98</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>roof repair company Cranston RI</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 06:26 UTC (cycle 31)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1373,6 +1373,62 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Statewide Plumbing &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>statewideplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://statewideplumbinginc.com/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>%20statewide.inc@verizon.net</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>(401) 944-5752</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Cranston RI</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>80</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>plumbing company Cranston RI</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 06:37 UTC (cycle 38)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1394,7 +1394,6 @@
           <t>https://statewideplumbinginc.com/</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>%20statewide.inc@verizon.net</t>
@@ -1424,6 +1423,62 @@
         </is>
       </c>
       <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Elite Mechanical</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>elitemechanicalpros.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://elitemechanicalpros.com/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>joey@elitemechanical406.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>406-256-1010</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Billings MT</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>80</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>HVAC contractor Billings MT</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 06:41 UTC (cycle 41)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1449,7 +1449,6 @@
           <t>https://elitemechanicalpros.com/</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>joey@elitemechanical406.com</t>
@@ -1479,6 +1478,66 @@
         </is>
       </c>
       <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Frontline Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>frontlineroofingllc.org</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://frontlineroofingllc.org/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Free Quote</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>frontlineroofingllc3@gmail.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(567) 702 0394</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Toledo OH</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>roofer Toledo OH</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 06:49 UTC (cycle 46)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1543,6 +1543,66 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Main Drain Cleaning Manchester, NH | Top Dog Sewer &amp; Drain</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>topdogsewer.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://www.topdogsewer.com/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Charlie Brennick</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>info@topdogsewer.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(603) 217-5209</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Manchester NH</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>94</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>drain cleaning service Manchester NH</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 06:50 UTC (cycle 47)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1603,6 +1603,62 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>P &amp; H Mechanical</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>pandhmechanical.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.pandhmechanical.com/</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>info@pandhmechanical.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>843-875-7675</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Summerville SC</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>100</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>furnace repair Summerville SC</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 06:52 UTC (cycle 48)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1624,7 +1624,6 @@
           <t>https://www.pandhmechanical.com/</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>info@pandhmechanical.com</t>
@@ -1654,6 +1653,66 @@
         </is>
       </c>
       <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>K-Ram Roofing Company Albuquerque</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>kramroofing.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://www.kramroofing.com/</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>What Happen</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>info@kramroofing.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>(505) 345-7663</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>98</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>residential roofing company Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 06:53 UTC (cycle 49)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1718,6 +1718,66 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Waldos Air Care</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>waldoac.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.waldoac.com/areas/springdale-ar</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Air Care</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>waldo@waldoac.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>(479) 405-4034</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Springdale AR</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>96</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>HVAC contractor Springdale AR</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 06:56 UTC (cycle 51)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1778,6 +1778,66 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Emergency Plumber Oxnard, CA 24/7 Plumbing Services</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>camarilloplumbingco.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://www.camarilloplumbingco.com/emergency-services/emergency-plumber-oxnard-ca</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>At Camarillo</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>info@camarilloplumbingco.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>(805) 482-8963</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Oxnard CA</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>100</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>emergency plumber Oxnard CA</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 06:59 UTC (cycle 53)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1838,6 +1838,62 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Surgi's Heating, Cooling &amp; Plumbing</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>surgisac.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://surgisac.com/plumbing/sewer-repair/</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>service@surgisac.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>(504) 215-7421</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>New Orleans LA</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>100</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>sewer repair New Orleans LA</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 07:08 UTC (cycle 59)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1859,7 +1859,6 @@
           <t>https://surgisac.com/plumbing/sewer-repair/</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>service@surgisac.com</t>
@@ -1889,6 +1888,62 @@
         </is>
       </c>
       <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Martin &amp; Sons LLC</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>martinandsons-stl.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.martinandsons-stl.com/st-louis/roofing</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>jason@kdinteractive.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>314-839-0700</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>St Louis MO</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>86</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>roof replacement St Louis MO</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 07:10 UTC (cycle 60)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1914,7 +1914,6 @@
           <t>https://www.martinandsons-stl.com/st-louis/roofing</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>jason@kdinteractive.com</t>
@@ -1944,6 +1943,62 @@
         </is>
       </c>
       <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Brecke - Cedar Rapids, IA | Family Legacy. Family Tradition.</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>brecke.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://brecke.com/excavation-services/sewer-and-water/</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>ben.brecht@brecke.com</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>(319) 396-7055</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Cedar Rapids IA</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>92</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>sewer repair Cedar Rapids IA</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 07:13 UTC (cycle 62)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1969,7 +1969,6 @@
           <t>https://brecke.com/excavation-services/sewer-and-water/</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>ben.brecht@brecke.com</t>
@@ -1999,6 +1998,66 @@
         </is>
       </c>
       <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Zees AirConditioning Inc</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>zeesairconditioninginc.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://zeesairconditioninginc.com/services/ac-repair-in-new-orleans/</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Abdelhamid Zaky</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>abdelhamid.zaky83@gmail.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>504-912-0490</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>New Orleans LA</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>100</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>air conditioning repair New Orleans LA</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 07:14 UTC (cycle 63)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2063,6 +2063,122 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Emergency Plumber Aberdeen, SD</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>aberdeen-sd.ldnplumbing.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://aberdeen-sd.ldnplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Aberdeen Sometimes</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>contact@ldnplumbing.com</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>(855) 804-9142</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>90</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>emergency plumber Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>C &amp; C Plumbing and Drain Cleaning</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>aberdeen-sd.ccplumbinganddrain.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://aberdeen-sd.ccplumbinganddrain.com/</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>contact@ccplumbinganddrain.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>(866) 547-4947</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>90</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>emergency plumber Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 07:16 UTC (cycle 64)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2144,7 +2144,6 @@
           <t>https://aberdeen-sd.ccplumbinganddrain.com/</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>contact@ccplumbinganddrain.com</t>
@@ -2174,6 +2173,66 @@
         </is>
       </c>
       <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Advantage Service Company</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>advantageserviceco.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://www.advantageserviceco.com/</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Little Rock</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>customerservice@advantageserviceco.com</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>(501) 663-2255</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Little Rock AR</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>100</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>heating and cooling company Little Rock AR</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 07:26 UTC (cycle 71)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2238,6 +2238,126 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Plumber in High Point, NC | Saunders Plumbing, INC</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>saundersplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://www.saundersplumbingservices.com/plumber-high-point-nc</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Saunders Plumbing</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>saundemi@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>(336) 629-8581</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>High Point NC</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>100</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>plumber High Point NC</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Maycon</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>callmaycon.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://callmaycon.com/roofing/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Star Service</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>maddie@callmaycon.com</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>(304) 208-8978</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Huntington WV</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>100</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Huntington WV</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 07:39 UTC (cycle 80)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2358,6 +2358,62 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>My Blog</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>plumbingansoniact.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://plumbingansoniact.com/areas-we-serve/waterbury/</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>support@plumbingansoniact.com</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>(207) 419-2600</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Waterbury CT</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>100</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>emergency plumber Waterbury CT</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 07:42 UTC (cycle 82)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2379,7 +2379,6 @@
           <t>https://plumbingansoniact.com/areas-we-serve/waterbury/</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>support@plumbingansoniact.com</t>
@@ -2409,6 +2408,66 @@
         </is>
       </c>
       <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Liberty RSC</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>libertyrsc.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://libertyrsc.com/roofing-carrollton</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Dallas County</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>info@libertyrsc.com</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>(469) 715-4603</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Carrollton TX</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>90</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>residential roofing company Carrollton TX</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 07:45 UTC (cycle 84)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2473,6 +2473,62 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Mapes Plumbing &amp; Heating | Plumbers | Rockford, IL</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>mapesplumbing.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://www.mapesplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>mapesplumbing@comcast.net</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>815-874-6533</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Rockford IL</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>96</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>plumbing company Rockford IL</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 07:48 UTC (cycle 86)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2494,7 +2494,6 @@
           <t>https://www.mapesplumbing.com/</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>mapesplumbing@comcast.net</t>
@@ -2524,6 +2523,66 @@
         </is>
       </c>
       <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Southwest Drain Doctors LLC</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>swfldraindoctors.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://www.swfldraindoctors.com/services/drain-cleaning-cape-coral-fl/</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Cape Coral</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>nick@swfldraindoctors.com</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>(239) 645-0857</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Cape Coral FL</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>100</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>drain cleaning service Cape Coral FL</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 07:49 UTC (cycle 87)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2588,6 +2588,62 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>HALEH ROOFING INC</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>halehroofinginc.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.halehroofinginc.com/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>hector@halehroofinginc.com</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>(818) 618-8919</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Santa Clarita CA</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>88</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>roofing contractor Santa Clarita CA</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 08:00 UTC (cycle 94)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2609,7 +2609,6 @@
           <t>https://www.halehroofinginc.com/</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>hector@halehroofinginc.com</t>
@@ -2639,6 +2638,122 @@
         </is>
       </c>
       <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Foley's Heating &amp; AC</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>foleysheating.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://foleysheating.com/</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>info@foleysheating.com</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>605.610.1840</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Sioux Falls SD</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>100</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>furnace repair Sioux Falls SD</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Ambassador Roofing &amp; Construction | Roofers | Edmond, OK</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ambassadorroofing.org</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://www.ambassadorroofing.org/</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Jay Shipp</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>heath@ambassadorconstruction.org</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>405-604-1002</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Edmond OK</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>72</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>roofer Edmond OK</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 08:03 UTC (cycle 96)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2664,7 +2664,6 @@
           <t>https://foleysheating.com/</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>info@foleysheating.com</t>
@@ -2754,6 +2753,62 @@
         </is>
       </c>
       <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ABC Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>abcmetalroofs.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://abcmetalroofs.com/</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>sales@abcmetalroofs.com</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>804-380-2504</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Richmond VA</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>92</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Richmond VA</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 08:06 UTC (cycle 98)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2779,7 +2779,6 @@
           <t>https://abcmetalroofs.com/</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>sales@abcmetalroofs.com</t>
@@ -2809,6 +2808,126 @@
         </is>
       </c>
       <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Best Coast Roofing</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>bestcoastroofing.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://www.bestcoastroofing.com/gresham-or-roof-replacement-and-repair</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>cody@bestcoastroofing.com</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>971.804.2207</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Gresham OR</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>90</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>roof repair company Gresham OR</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Roofing Services in Gresham, OR - Riley Roofing</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>rileyroofingnw.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://rileyroofingnw.com/service-areas/gresham-or</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Roof Replacements</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>paige@rileyroofingnw.com</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>(971) 997-2112</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Gresham OR</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>90</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>roof repair company Gresham OR</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 08:07 UTC (cycle 99)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2933,6 +2933,62 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Orlando, FL Plumber</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>plumbingorlandofl.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://plumbingorlandofl.com/water-heater-repair/</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>hello@plumbingorlandofl.com</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>689 220 2023</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Orlando FL</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>76</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>water heater repair Orlando FL</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 08:09 UTC (cycle 100)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2954,7 +2954,6 @@
           <t>https://plumbingorlandofl.com/water-heater-repair/</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>hello@plumbingorlandofl.com</t>
@@ -2984,6 +2983,66 @@
         </is>
       </c>
       <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>jaguarheatingandair.com</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>jaguarheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://www.jaguarheatingandair.com/heat-pump/heat-pump-installation-sacramento-ca</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Knowing When</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>jaguarheatingandair@gmail.com</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>916-646-2007</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Sacramento CA</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>90</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>heat pump installation Sacramento CA</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 08:21 UTC (cycle 108)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3048,6 +3048,66 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Kinnee Brothers Roofing</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>kinneebrosroofing.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://www.kinneebrosroofing.com/</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Drew Kinnee</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>info@kinneebrosroofing.com</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>412-844-5999</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>90</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>roofing contractor Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 08:35 UTC (cycle 118)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3108,6 +3108,62 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Home | McCalls HVAC</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>mccallshvac.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://www.mccallshvac.com/</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Company Name</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>office.mccalls@gmail.com</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Savannah GA</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>76</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>HVAC contractor Savannah GA</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 08:47 UTC (cycle 126)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3139,7 +3139,6 @@
           <t>office.mccalls@gmail.com</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>Savannah GA</t>
@@ -3159,6 +3158,62 @@
         </is>
       </c>
       <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Cool Sunshine Heating &amp; Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>cool-sunshine.com</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://www.cool-sunshine.com/</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>info@cool-sunshine.com</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>303-287-1846</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Denver CO</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>90</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>heating and cooling company Denver CO</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 08:53 UTC (cycle 130)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3184,7 +3184,6 @@
           <t>https://www.cool-sunshine.com/</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>info@cool-sunshine.com</t>
@@ -3214,6 +3213,66 @@
         </is>
       </c>
       <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>A/C Maintenance &amp; Repair | Honolulu, HI | Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>airconditioningexpertshi.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://www.airconditioningexpertshi.com/repair-maintenance</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Maintenance About</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>airconditioningexpertshi@gmail.com</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>(808) 732-2236</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Honolulu HI</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>86</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>air conditioning repair Honolulu HI</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 08:56 UTC (cycle 132)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3278,6 +3278,186 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Abilene Roof Pros</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>abileneroofpros.com</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://www.abileneroofpros.com/</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Roof Pros</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>contact@abileneroofpros.com</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>(325) 400-2861</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Abilene TX</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>98</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>roof replacement Abilene TX</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Paterson Plumbing Pros</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>patersonplumbingpros.com</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://patersonplumbingpros.com/</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Paterson Plumbing</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>info@patersonplumbingpros.com</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>(973) 577-6890</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Paterson NJ</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>90</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>plumber Paterson NJ</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation &amp; Replacement | Dunedin &amp; Clearwater, FL</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>coolwizardairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://coolwizardairconditioning.com/heat-pump-installation-replacement/</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Serviceg Since</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>info@coolwizardac.com</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>(727) 542-6178</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Clearwater FL</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>90</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>heat pump installation Clearwater FL</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 08:58 UTC (cycle 133)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3458,6 +3458,62 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>HeatPumps NorthWest</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>heatpumpnorthwest.com</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://www.heatpumpnorthwest.com/heat-pump-installation-salem/</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>northwest@info.com</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>(503) 303-7420</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Salem OR</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>100</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>heat pump installation Salem OR</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 09:11 UTC (cycle 142)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3479,7 +3479,6 @@
           <t>https://www.heatpumpnorthwest.com/heat-pump-installation-salem/</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
           <t>northwest@info.com</t>
@@ -3509,6 +3508,122 @@
         </is>
       </c>
       <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Frank's Cooling and Heating LLC</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>franktheacguy.com</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://www.franktheacguy.com/</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>info@franktheacguy.com</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>(520) 612-3388</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Tucson AZ</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>100</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>HVAC contractor Tucson AZ</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Metal Roofing Services Milwaukee, WI</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>milwaukee-wi.dans-roofing.com</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://milwaukee-wi.dans-roofing.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Energy Savings</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>info@dans-roofing.com</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>(888) 766-0591</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Milwaukee WI</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>90</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Milwaukee WI</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 09:18 UTC (cycle 147)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3534,7 +3534,6 @@
           <t>https://www.franktheacguy.com/</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
           <t>info@franktheacguy.com</t>
@@ -3624,6 +3623,122 @@
         </is>
       </c>
       <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>HVAC Contractor in Mesquite, TX</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>misterairrepair.com</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://www.misterairrepair.com/service-areas/mesquite-tx</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>customer@misterairrepair.com</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>972-556-5969</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Mesquite TX</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>100</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>HVAC contractor Mesquite TX</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Air Conditioning Repair and Heating Rowlett, TX</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>5starhvaccontractors.com</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://5starhvaccontractors.com/service-area/mesquite-hvac/</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Upgrade Your</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>support@5starhvaccontractors.com</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>972-845-1103</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Mesquite TX</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>100</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>HVAC contractor Mesquite TX</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 09:24 UTC (cycle 151)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3649,7 +3649,6 @@
           <t>https://www.misterairrepair.com/service-areas/mesquite-tx</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>customer@misterairrepair.com</t>
@@ -3739,6 +3738,66 @@
         </is>
       </c>
       <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>619 Heating and Air</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>619heatingandair.com</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://619heatingandair.com/</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Message An</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>619heatingandair@gmail.com</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>(619) 616-5538</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Chula Vista CA</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>86</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>HVAC contractor Chula Vista CA</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 09:33 UTC (cycle 157)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3803,6 +3803,182 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Peli Plumbing</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>peliplumbing.com</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://peliplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Softeners Water</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>office@peliplumbing.com</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>909-485-2110</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Rancho Cucamonga CA</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>100</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>plumbing company Rancho Cucamonga CA</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>TEO Roofing</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>teoroofing.com</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://www.teoroofing.com/</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>teo@teoroofing.com</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>(301) 466-3630</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Frederick MD</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>90</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>roofer Frederick MD</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>ETC Services LLC Roofing Specialists</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>etcroofing.com</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://etcroofing.com/</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Owner Jason</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>info@etcservices.com</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2705169780</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Frederick MD</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>78</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>roofer Frederick MD</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 09:36 UTC (cycle 159)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3884,7 +3884,6 @@
           <t>https://www.teoroofing.com/</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
           <t>teo@teoroofing.com</t>
@@ -3974,6 +3973,66 @@
         </is>
       </c>
       <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Roger’s Plumbing</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>callrogersplumbing.com</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://callrogersplumbing.com/round-rock-tx/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Service Makes</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>service@callrogersplumbing.com</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>(737) 285-4346</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Round Rock TX</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>90</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>drain cleaning service Round Rock TX</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 09:38 UTC (cycle 160)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4038,6 +4038,62 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Thermex Valley</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>thermexvalley.com</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://thermexvalley.com/</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>thermex01@yakima.net</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>(509) 965-0630</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Yakima WA</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>90</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>heating and cooling company Yakima WA</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 09:39 UTC (cycle 161)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4059,7 +4059,6 @@
           <t>https://thermexvalley.com/</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
           <t>thermex01@yakima.net</t>
@@ -4089,6 +4088,62 @@
         </is>
       </c>
       <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Drain Cleaning Service Tucson AZ | Plumber Kings</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>theplumberkings.com</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://theplumberkings.com/services/drain-cleaning</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>theplumberkings@gmail.com</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>(520) 777-0546</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Tucson AZ</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>90</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>drain cleaning service Tucson AZ</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 09:47 UTC (cycle 166)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4114,7 +4114,6 @@
           <t>https://theplumberkings.com/services/drain-cleaning</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
           <t>theplumberkings@gmail.com</t>
@@ -4144,6 +4143,66 @@
         </is>
       </c>
       <c r="L64" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>ASAP Service Plumbing LLC</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>asapserviceplumbing.com</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://asapserviceplumbing.com/emergency-plumber-in-kissimmee/</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Osceola County</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>service@asapserviceplumbing.com</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>(407) 565 8808</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Kissimmee FL</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>100</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>emergency plumber Kissimmee FL</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 09:50 UTC (cycle 168)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4208,6 +4208,126 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Sewer Line Repair | In-Ground Repairs | San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>drainbustersplumbing.net</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://www.drainbustersplumbing.net/sewer-line-repair</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Drain Busters</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>dbp.khano@gmail.com</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>(650) 419-0806</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>San Francisco CA</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>100</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>sewer repair San Francisco CA</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Five Star Plumbing &amp; Rooter - San Francisco's Family Plumber — Honest Pricing, E</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>fivestarplumbingsf.com</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://fivestarplumbingsf.com/services/sewer-line-repair/</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>events@tommygatzent.com</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>(415) 724-7083</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>San Francisco CA</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>90</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>sewer repair San Francisco CA</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 09:57 UTC (cycle 173)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4328,6 +4328,66 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Trinity Heating and Air</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>trinityheatingair.com</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://trinityheatingair.com/locations/elk-grove/</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Andrew Mitchell</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>trinityheatingandairca@gmail.com</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>(279) 667-4304</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Elk Grove CA</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>90</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>HVAC contractor Elk Grove CA</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 09:59 UTC (cycle 174)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4388,6 +4388,66 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Dependable Roofing and Solar Cleaning</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>getdependableroofing.com</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://www.getdependableroofing.com/</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Owners Get</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>example@mysite.com</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>(520) 444-3180</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Tucson AZ</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>100</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>roofing contractor Tucson AZ</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 10:13 UTC (cycle 184)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4448,6 +4448,62 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Warrior Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>warriorhca.com</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://warriorhca.com/services/heating-repair</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>warriorhca@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>(205) 371-6556</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Tuscaloosa AL</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>90</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>furnace repair Tuscaloosa AL</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 10:29 UTC (cycle 195)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L70"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4469,7 +4469,6 @@
           <t>https://warriorhca.com/services/heating-repair</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
           <t>warriorhca@yahoo.com</t>
@@ -4499,6 +4498,126 @@
         </is>
       </c>
       <c r="L70" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Premier AC &amp; Heating LLC</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>premieracandheating.com</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://www.premieracandheating.com/</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Rock Hill</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>premierac@comporium.net</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>(803) 366-8024</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Rock Hill SC</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>90</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>AC installation Rock Hill SC</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>AC Installation in Rock Hill, SC | Carolina Refrigeration</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>crcoolingandheating.com</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://www.crcoolingandheating.com/air-conditioning-installation</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Button How</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>carolinarefrigeration@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>803-902-3695</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Rock Hill SC</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>90</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>AC installation Rock Hill SC</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 10:31 UTC (cycle 196)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4623,6 +4623,66 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>24/7 Emergency Plumber in San Marcos, TX</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>emergencyplumbersanmarcos.net</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://emergencyplumbersanmarcos.net/</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Plumber San</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>info@emergencyplumbersanmarcos.net</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>(512) 592-1981</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>San Marcos TX</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>90</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>emergency plumber San Marcos TX</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 16:38 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L73"/>
+  <dimension ref="A1:L74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4683,6 +4683,66 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>HVAC Installation Pro</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>hvacinstallationpro.com</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://hvacinstallationpro.com/location/hvac-southaven-ms.html</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Installation Pro</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>info@hvacinstallationpro.com</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>(888) 217-8434</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Southaven MS</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>90</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>heat pump installation Southaven MS</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 16:39 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L74"/>
+  <dimension ref="A1:L75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4743,6 +4743,66 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Roofing Contractor Franklin TN | Roof Commander</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>roofcommander.net</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://www.roofcommander.net/areas/franklin</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Roof Commander</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>chad@roofcommander.net</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>(615) 218-6872</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Franklin TN</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>90</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>roofing contractor Franklin TN</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 16:42 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L75"/>
+  <dimension ref="A1:L76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4803,6 +4803,66 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>SureSealContractors</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>suresealcontractors.com</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://www.suresealcontractors.com/</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Room Additions</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>example@mysite.com</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>(812) 219-9629</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Bloomington IN</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>100</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>roofer Bloomington IN</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 16:51 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:L79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4863,6 +4863,182 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Roof Tech Contractors</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>rooftechcontractors.com</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://www.rooftechcontractors.com/roofing/myrtle-beach-sc</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Roof Tec</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>contactus@rooftechcontractors.com</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>(843)331-1166</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Myrtle Beach SC</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>100</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>roofing contractor Myrtle Beach SC</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Response Roofing</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>responseroofingsc.com</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://responseroofingsc.com/</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>South Carolina</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>responseroofingsc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>(854) 894-2128</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Myrtle Beach SC</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>90</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>roofing contractor Myrtle Beach SC</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Metal Roofing &amp; Siding Services | RVM All Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>rvmallmetalroofing.com</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://rvmallmetalroofing.com/</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>info@rvmallmetalroofing.com</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>360.224.4052</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Bellingham WA</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>90</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Bellingham WA</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 16:55 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L79"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5004,7 +5004,6 @@
           <t>https://rvmallmetalroofing.com/</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
           <t>info@rvmallmetalroofing.com</t>
@@ -5034,6 +5033,66 @@
         </is>
       </c>
       <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Emergency Leak Detection | CG Plumbing | El Dorado Co.</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>cgplumbingservice.com</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://www.cgplumbingservice.com/emergency-leak-detection</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>El Dorado</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>chrisgraubart@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>916-413-2480</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Elk Grove CA</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>100</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>emergency plumber Elk Grove CA</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 16:57 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5098,6 +5098,66 @@
         </is>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Air Temp Mechanical Services | Comprehensive HVAC Solutions</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>ctairtemp.com</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://ctairtemp.com/</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Jeff Leone</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>atmsinfo@ctairtemp.com</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>860.953.8888</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Hartford CT</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>98</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>HVAC contractor Hartford CT</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 17:01 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L81"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5158,6 +5158,66 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Olde Arva Plumbing</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>emergencyplumbersarvadaco.com</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://emergencyplumbersarvadaco.com/service-areas/pueblo-co/</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Olde Arva</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>oldearva@gmail.com</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>(720) 905-4004</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Pueblo CO</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>90</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>emergency plumber Pueblo CO</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 17:03 UTC (cycle 18)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5218,6 +5218,66 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>PEY Roofing</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>peyroofing.com</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://peyroofing.com/location/moreno-valley/</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>John Smith</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>peyroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>(424) 424-2202</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Moreno Valley CA</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>90</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>residential roofing company Moreno Valley CA</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 17:10 UTC (cycle 23)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L83"/>
+  <dimension ref="A1:L84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5278,6 +5278,66 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Hoosier Indoor Air</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>hoosierindoorair.com</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://hoosierindoorair.com/service-areas/carmel/ac-repair/</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Indoor Air</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>service@hoosierindoorair.com</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>317-466-7437</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Carmel IN</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>100</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>air conditioning repair Carmel IN</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 17:19 UTC (cycle 29)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5338,6 +5338,182 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Killeen hvac repair</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>killeenhvacrepair.com</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://killeenhvacrepair.com/killeen-ac-repair/</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Mike Smith</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>info@killeenhvacrepair.com</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>(254) 123-4567</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Killeen TX</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>100</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>air conditioning repair Killeen TX</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Residential AC Installation | Home AC Systems | Pasadena, TX</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>absolutevalueacllctx.com</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://www.absolutevalueacllctx.com/residential-ac-installation</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Absolute Value</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>service@absolutevalueair.com</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>(281) 670-8232</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>96</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>AC installation Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>AC Repair &amp; Installation Pasadena TX</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>acrepairpasadenatx.com</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://acrepairpasadenatx.com/</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>service@acrepairpasadenatx.com</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>713-588-9309</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>84</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>AC installation Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 17:36 UTC (cycle 41)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:L88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5479,7 +5479,6 @@
           <t>https://acrepairpasadenatx.com/</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
           <t>service@acrepairpasadenatx.com</t>
@@ -5509,6 +5508,62 @@
         </is>
       </c>
       <c r="L87" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Metal Hero</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>metalhero.com</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://www.metalhero.com/</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>ray@metalhero.com</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>504-470-8609</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Metairie LA</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>80</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Metairie LA</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 17:45 UTC (cycle 47)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5534,7 +5534,6 @@
           <t>https://www.metalhero.com/</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
           <t>ray@metalhero.com</t>
@@ -5564,6 +5563,122 @@
         </is>
       </c>
       <c r="L88" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Roofing Contractor in Torrance, CA</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>summerroofinginc.com</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://www.summerroofinginc.com/area-we-serve/roofing-contractor-in-torrance-ca</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Repair Versus</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>cesar@summerroofinginc.com</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>760-571-1040</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Torrance CA</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>90</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>roofing contractor Torrance CA</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Stamford, CT</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>advancedbasementct.com</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://www.advancedbasementct.com/stamford-ct-sewer-line-install-repair-and-replacement/</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>brian@advancedbasementct.com</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>(203) 274-8802</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Stamford CT</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>74</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>sewer repair Stamford CT</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 18:02 UTC (cycle 59)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L90"/>
+  <dimension ref="A1:L92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5649,7 +5649,6 @@
           <t>https://www.advancedbasementct.com/stamford-ct-sewer-line-install-repair-and-replacement/</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
           <t>brian@advancedbasementct.com</t>
@@ -5679,6 +5678,122 @@
         </is>
       </c>
       <c r="L90" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Piper Plumbing</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>piperplumbing.com</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://piperplumbing.com/garland/emergency-plumbing/</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Years Experience</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>service@piperplumbing.com</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>214-467-9091</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Garland TX</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>90</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>emergency plumber Garland TX</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>24 Hour Emergency Plumber in Garland, TX</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>emergencyplumbergarland.com</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://emergencyplumbergarland.com/</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>admin@predictiveyield.com</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>469-972-8600</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Garland TX</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>90</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>emergency plumber Garland TX</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 18:10 UTC (cycle 64)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L92"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5764,7 +5764,6 @@
           <t>https://emergencyplumbergarland.com/</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
           <t>admin@predictiveyield.com</t>
@@ -5794,6 +5793,66 @@
         </is>
       </c>
       <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Roofer Grand Island, NE | L6 Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>l6contracting.com</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://www.l6contracting.com/</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Frequently Asked</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>jerry@l6contracting.com</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>(308) 390-2830</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Grand Island NE</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>100</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>roofer Grand Island NE</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 18:16 UTC (cycle 68)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L93"/>
+  <dimension ref="A1:L94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5858,6 +5858,62 @@
         </is>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Roof Replacement in Medford</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>allweatherroofingandconst.com</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://allweatherroofingandconst.com/locations/medford-or/roof-replacement</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>info@allweatherroofingandconst.com</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>(866) 700-3860</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Medford OR</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>90</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>roof replacement Medford OR</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 18:19 UTC (cycle 70)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L94"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5879,7 +5879,6 @@
           <t>https://allweatherroofingandconst.com/locations/medford-or/roof-replacement</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
           <t>info@allweatherroofingandconst.com</t>
@@ -5909,6 +5908,62 @@
         </is>
       </c>
       <c r="L94" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>The Red Shirt Guys Roofing</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>theredshirtguys.com</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://theredshirtguys.com/</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>info@theredshirtguys.com</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>803.243.3968</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Columbia SC</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>96</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>residential roofing company Columbia SC</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 18:33 UTC (cycle 80)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5934,7 +5934,6 @@
           <t>https://theredshirtguys.com/</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
           <t>info@theredshirtguys.com</t>
@@ -5964,6 +5963,66 @@
         </is>
       </c>
       <c r="L95" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Noble Roofing</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>nobleroofing.co</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://nobleroofing.co/locations/conroe-tx/residential/</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Noble Roofing</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>contact@nobleroofing.co</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>(346) 496-4500</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Conroe TX</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>100</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>residential roofing company Conroe TX</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 18:45 UTC (cycle 88)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L96"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6028,6 +6028,62 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>CEC Plumbing</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>cecplumbing.com</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://cecplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>support@cecplumbing.com</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>301-259-1475</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Champaign IL</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>90</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>plumbing company Champaign IL</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 18:49 UTC (cycle 91)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L97"/>
+  <dimension ref="A1:L98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6049,7 +6049,6 @@
           <t>https://cecplumbing.com/</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
           <t>support@cecplumbing.com</t>
@@ -6079,6 +6078,66 @@
         </is>
       </c>
       <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>A&amp;A HVAC LLC</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>aahvacrgv.com</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://www.aahvacrgv.com/services/heating-repair</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Rio Grande</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>info@aahvacrgv.com</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>(877) 237-1820</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>McAllen TX</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>90</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>furnace repair McAllen TX</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 18:57 UTC (cycle 96)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L98"/>
+  <dimension ref="A1:L99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6143,6 +6143,66 @@
         </is>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Austin Roof Repair</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>roofrepairaustin.net</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://roofrepairaustin.net/</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Sarah Johnson</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>info@roofrepairaustin.net</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>512-861-0303</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Austin TX</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>90</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>roof repair company Austin TX</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 19:05 UTC (cycle 102)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L99"/>
+  <dimension ref="A1:L100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6203,6 +6203,62 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Grimes Mechanical</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>grimesmechanicalcompany.com</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://www.grimesmechanicalcompany.com/</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>support@grimescorp.com</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>(385) 423-2657</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Ogden UT</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>90</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>HVAC contractor Ogden UT</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 19:07 UTC (cycle 103)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6224,7 +6224,6 @@
           <t>https://www.grimesmechanicalcompany.com/</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
           <t>support@grimescorp.com</t>
@@ -6254,6 +6253,66 @@
         </is>
       </c>
       <c r="L100" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Roofing Contractor in Clearwater, FL</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>clearwaterflroofingpros.com</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://clearwaterflroofingpros.com/</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Pinellas County</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>bloomingdaleproductions@gmail.com</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>(727) 594-0974</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Clearwater FL</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>100</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>roofing contractor Clearwater FL</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 19:09 UTC (cycle 104)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6318,6 +6318,122 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Water Heater Installation and Repair | Bakersfield, CA</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>topgradeplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://www.topgradeplumbinginc.com/water-heater-installation-and-repair</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>edgar@topgradeplumbing.services</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>(661) 214-8048</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Bakersfield CA</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>94</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>water heater repair Bakersfield CA</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>chapmansborohvacservice.com</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>chapmansborohvacservice.com</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://chapmansborohvacservice.com/locations/clarksville-tn-furnace-repair</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Local Climate</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>info@chapmansborohvacservice.com</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>(931) 354-5956</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Clarksville TN</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>90</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>furnace repair Clarksville TN</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 19:20 UTC (cycle 112)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L103"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6339,7 +6339,6 @@
           <t>https://www.topgradeplumbinginc.com/water-heater-installation-and-repair</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
           <t>edgar@topgradeplumbing.services</t>
@@ -6429,6 +6428,66 @@
         </is>
       </c>
       <c r="L103" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Roofs R Us</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>roofsrusminnesota.com</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://roofsrusminnesota.com/service-areas/brooklyn-park</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Twin Cities</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>estimates@roofsrusminnesota.com</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>(763) 762-9031</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Brooklyn Park MN</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>100</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>roof replacement Brooklyn Park MN</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 19:22 UTC (cycle 113)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6493,6 +6493,66 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>HVAC Company New Jersey</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>ac-installation-woodbridge.aeshvacnj.com</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://ac-installation-woodbridge.aeshvacnj.com/</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Call Us</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>example@mail.com</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>(888) 978-1291</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>100</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>AC installation Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 19:23 UTC (cycle 114)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6553,6 +6553,66 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Laredo, TX 78041-6840</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>ferguson.com</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://www.ferguson.com/store/tx/laredo/plumbingpvf-1160</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>All Website</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>customer.support@ferguson.com</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>956-284-2393</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Laredo TX</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>100</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>water heater repair Laredo TX</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 19:44 UTC (cycle 128)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L106"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6613,6 +6613,62 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Heat Pump in Pittsburgh, PA | Sta So Cool HVAC</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>stasocoolhvac.com</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://www.stasocoolhvac.com/pittsburgh-pa-heat-pumps</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>stasocoolhvac@gmail.com</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>(412) 290-4980</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>90</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>heat pump installation Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 19:45 UTC (cycle 129)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6634,7 +6634,6 @@
           <t>https://www.stasocoolhvac.com/pittsburgh-pa-heat-pumps</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
           <t>stasocoolhvac@gmail.com</t>
@@ -6664,6 +6663,66 @@
         </is>
       </c>
       <c r="L107" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Smart Choice Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>mysmartchoiceac.com</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://mysmartchoiceac.com/heat-pump-installation/</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Star Rated</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>info@choosesmartchoice.com</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>(210) 367-0908</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>San Antonio TX</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>100</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>heat pump installation San Antonio TX</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 19:47 UTC (cycle 130)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L108"/>
+  <dimension ref="A1:L109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6728,6 +6728,66 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Hernandez Roofing Pros</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>hernandezroofingpros.com</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://hernandezroofingpros.com/silver-spring-roofing/</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Network Helping</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>hernandezcompany1@gmail.com</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>(240) 479-6948</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Silver Spring MD</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>100</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>roof repair company Silver Spring MD</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 19:56 UTC (cycle 136)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L109"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6788,6 +6788,62 @@
         </is>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Pipe Doctor — Licensed Master Plumber | Toledo &amp; NW Ohio</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>pipedrhelp.com</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://www.pipedrhelp.com/</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>pipedrwagner@gmail.com</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>419-887-2833</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Toledo OH</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>88</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>plumber Toledo OH</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 20:00 UTC (cycle 139)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L110"/>
+  <dimension ref="A1:L111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6809,7 +6809,6 @@
           <t>https://www.pipedrhelp.com/</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
           <t>pipedrwagner@gmail.com</t>
@@ -6839,6 +6838,66 @@
         </is>
       </c>
       <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Roofing Contractor Columbus OH</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>supremeexterior.com</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://supremeexterior.com/</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Owens Corning</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>info@supremeexterior.com</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>(614) 517-1717</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Columbus OH</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>90</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>roofing contractor Columbus OH</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 20:04 UTC (cycle 142)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L111"/>
+  <dimension ref="A1:L113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6903,6 +6903,122 @@
         </is>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Southern California Mechanical</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>southerncaliforniamechanical.com</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://southerncaliforniamechanical.com/</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>scmechanical@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>(661) 361-3401</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Palmdale CA</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>100</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>HVAC contractor Palmdale CA</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>DAC Heating &amp; Air | HVAC Services in Palmdale, CA</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>dachvac.com</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://www.dachvac.com/</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Family You</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>info@dachvac.com</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>(661) 441-2787</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Palmdale CA</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>86</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>HVAC contractor Palmdale CA</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 20:07 UTC (cycle 144)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L113"/>
+  <dimension ref="A1:L115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6924,7 +6924,6 @@
           <t>https://southerncaliforniamechanical.com/</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
           <t>scmechanical@yahoo.com</t>
@@ -7014,6 +7013,122 @@
         </is>
       </c>
       <c r="L113" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Urban Plumbing Co</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>uplumbingco.com</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://www.uplumbingco.com/</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>office@uplumbingco.com</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>804-625-5557</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Richmond VA</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>94</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>plumbing company Richmond VA</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Precision Roofing Alabama</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>precisionroofingalabama.com</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://www.precisionroofingalabama.com/montgomery</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Roofs Completed</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>contact.precisionral@gmail.com</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>(334) 318-7255</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Montgomery AL</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>90</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>roofing contractor Montgomery AL</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 20:09 UTC (cycle 145)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L115"/>
+  <dimension ref="A1:L116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7039,7 +7039,6 @@
           <t>https://www.uplumbingco.com/</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
           <t>office@uplumbingco.com</t>
@@ -7129,6 +7128,66 @@
         </is>
       </c>
       <c r="L115" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Saldana Roofing</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>saldanaroofing.org</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://saldanaroofing.org/</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Johnson City</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>saldanaroofing04@gmail.com</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>(423) 767-3390</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Johnson City TN</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>90</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>roofing contractor Johnson City TN</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 20:10 UTC (cycle 146)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L116"/>
+  <dimension ref="A1:L117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7193,6 +7193,62 @@
         </is>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Phoenix Roofing Company | AZ Roofing LLC | Get an Estimate</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>azroofllc.com</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://azroofllc.com/service-areas/phoenix-az</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>alex@azroofllc.com</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>6029991333</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>88</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>residential roofing company Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 20:21 UTC (cycle 153)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L117"/>
+  <dimension ref="A1:L118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7214,7 +7214,6 @@
           <t>https://azroofllc.com/service-areas/phoenix-az</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
           <t>alex@azroofllc.com</t>
@@ -7244,6 +7243,66 @@
         </is>
       </c>
       <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Air Support Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>airsupportky.com</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://airsupportky.com/furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Helpful Tips</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>office@airsupportky.com</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>502-771-8179</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Louisville KY</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>100</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>furnace repair Louisville KY</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 20:22 UTC (cycle 154)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L118"/>
+  <dimension ref="A1:L120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7308,6 +7308,126 @@
         </is>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Alexander Plumbing</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>alexanderplumbingcontractor.com</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://alexanderplumbingcontractor.com/</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Chicagoland Area</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>patricksakolari@ameritech.net</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>(847) 742-0541</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Elgin IL</t>
+        </is>
+      </c>
+      <c r="I119" t="n">
+        <v>100</v>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>plumber Elgin IL</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Midwest Roofing Solutions LLC | Expert Roofing &amp; Storm Repair in Kansas City</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>midwestroofingsolutionskc.com</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://midwestroofingsolutionskc.com/</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Google Bryan</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>jeff@midwestroofingsolutionskc.com</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>(913)-379-7290</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Olathe KS</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>90</v>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>roof repair company Olathe KS</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 20:24 UTC (cycle 155)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L120"/>
+  <dimension ref="A1:L121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7428,6 +7428,66 @@
         </is>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Roofing, Roofing Company, Roofers &amp; Roof Repair</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>therooferdirect.com</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://www.therooferdirect.com/service-areas/columbia-sc/</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Repair Commercial</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>robertburnam@att.net</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>(855) 338-7663</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Columbia SC</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>90</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>roof replacement Columbia SC</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 20:31 UTC (cycle 160)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L121"/>
+  <dimension ref="A1:L122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7488,6 +7488,66 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Roof Medic</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>roofmedic.com</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>https://roofmedic.com/roof-repair/</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Message From</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>contact@roofmedic.com</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>704.228.7788</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Charlotte NC</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>100</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>roof repair company Charlotte NC</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 20:38 UTC (cycle 165)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L122"/>
+  <dimension ref="A1:L123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7548,6 +7548,62 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Icon Mechanical Inc.</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>iconmechanicalinc.com</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>https://www.iconmechanicalinc.com/</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>office@iconmechanicalinc.com</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>623-386-7804</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>90</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>HVAC contractor Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 20:41 UTC (cycle 167)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L123"/>
+  <dimension ref="A1:L124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7569,7 +7569,6 @@
           <t>https://www.iconmechanicalinc.com/</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
           <t>office@iconmechanicalinc.com</t>
@@ -7599,6 +7598,62 @@
         </is>
       </c>
       <c r="L123" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Free Flow Sewer &amp; Drain Solutions</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>freeflow307.com</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>https://freeflow307.com/</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>tyler.freeflow@gmail.com</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>307-460-8985</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Laramie WY</t>
+        </is>
+      </c>
+      <c r="I124" t="n">
+        <v>84</v>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>drain cleaning service Laramie WY</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 20:46 UTC (cycle 170)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L124"/>
+  <dimension ref="A1:L126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7624,7 +7624,6 @@
           <t>https://freeflow307.com/</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr">
         <is>
           <t>tyler.freeflow@gmail.com</t>
@@ -7654,6 +7653,122 @@
         </is>
       </c>
       <c r="L124" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Emergency Plumber in Wichita, KS – 24 Hour Plumbing Service Near You</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>wichitaemergencyplumber.com</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>https://www.wichitaemergencyplumber.com/</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>contact@wichitaemergencyplumber.com</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>855-785-3024</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Wichita KS</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>100</v>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>emergency plumber Wichita KS</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Vector Services</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>callvector.com</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>https://callvector.com/</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Hennepin County</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>service@callvector.com</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>651-447-7776</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>90</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>HVAC contractor Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 20:50 UTC (cycle 173)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L126"/>
+  <dimension ref="A1:L127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7679,7 +7679,6 @@
           <t>https://www.wichitaemergencyplumber.com/</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
       <c r="F125" t="inlineStr">
         <is>
           <t>contact@wichitaemergencyplumber.com</t>
@@ -7769,6 +7768,66 @@
         </is>
       </c>
       <c r="L126" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>New Roofing | Dayton, OH | Dahm Brothers Co. Inc.</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>dahmbrothersroofing.com</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>https://www.dahmbrothersroofing.com/</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Chris Dahm</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>dahmbrothers@dahmbrothersroofing.com</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>(937) 461-5627</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Dayton OH</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>100</v>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>residential roofing company Dayton OH</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 20:56 UTC (cycle 177)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L127"/>
+  <dimension ref="A1:L128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7833,6 +7833,66 @@
         </is>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>ROOFING TYLER TX LLC | Residential and Commercial Roofers</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>roofingtylertxpro.com</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>https://roofingtylertxpro.com/</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Installation Patio</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>b.wagner@sprayfoam-roofing.com</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>(903) 560-4072</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Tyler TX</t>
+        </is>
+      </c>
+      <c r="I128" t="n">
+        <v>100</v>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>roofer Tyler TX</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 20:58 UTC (cycle 178)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L128"/>
+  <dimension ref="A1:L129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7893,6 +7893,62 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Taylor Plumbing</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>taylorplumbing.net</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>https://taylorplumbing.net/</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>info@taylorplumbing.net</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>440-635-0642</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Cleveland OH</t>
+        </is>
+      </c>
+      <c r="I129" t="n">
+        <v>86</v>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>plumbing company Cleveland OH</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 21:11 UTC (cycle 187)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L129"/>
+  <dimension ref="A1:L131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7914,7 +7914,6 @@
           <t>https://taylorplumbing.net/</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr">
         <is>
           <t>info@taylorplumbing.net</t>
@@ -7944,6 +7943,118 @@
         </is>
       </c>
       <c r="L129" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Emergency Plumber in Franklin, TN | 24/7 Plumbing Services</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>expressplumberfranklin.com</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>https://expressplumberfranklin.com/</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>contact@expressplumberfranklin.com</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>(615) 616-0512</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Franklin TN</t>
+        </is>
+      </c>
+      <c r="I130" t="n">
+        <v>90</v>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>emergency plumber Franklin TN</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Wright Choice Plumbing</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>callwrightchoiceplumbing.com</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>https://callwrightchoiceplumbing.com/services/sewer-line-repair/</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>jacob@wrightchoiceplumbing.com</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>(336) 991-0670</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>High Point NC</t>
+        </is>
+      </c>
+      <c r="I131" t="n">
+        <v>90</v>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>sewer repair High Point NC</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 21:15 UTC (cycle 190)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L131"/>
+  <dimension ref="A1:L132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7969,7 +7969,6 @@
           <t>https://expressplumberfranklin.com/</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr">
         <is>
           <t>contact@expressplumberfranklin.com</t>
@@ -8025,7 +8024,6 @@
           <t>https://callwrightchoiceplumbing.com/services/sewer-line-repair/</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr">
         <is>
           <t>jacob@wrightchoiceplumbing.com</t>
@@ -8055,6 +8053,66 @@
         </is>
       </c>
       <c r="L131" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Dutton Plumbing Inc - Bloomington, Indiana</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>duttonplumbing.org</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>https://www.duttonplumbing.org/service-areas/bloomington-indiana</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Dutton Plumbing</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>duttonplumbinginc@outlook.com</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>(812) 447-7881</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Bloomington IN</t>
+        </is>
+      </c>
+      <c r="I132" t="n">
+        <v>80</v>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>plumbing company Bloomington IN</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-28 21:20 UTC (cycle 193)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L132"/>
+  <dimension ref="A1:L133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8118,6 +8118,66 @@
         </is>
       </c>
     </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>HelloCool AC Repairs</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>hellocoolacrepairs.com</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>https://hellocoolacrepairs.com/hvac-in-hollywood-fl/</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Team The</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>info@hellocoolacrepairs.com</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>(786) 947-6278</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Hollywood FL</t>
+        </is>
+      </c>
+      <c r="I133" t="n">
+        <v>90</v>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>HVAC contractor Hollywood FL</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 21:29 UTC (cycle 199)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L133"/>
+  <dimension ref="A1:L134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8178,6 +8178,66 @@
         </is>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>PLUMBING SEWER &amp; DRAIN SERVICE</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>plumbingsewerdrainservice.com</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>https://plumbingsewerdrainservice.com/</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Staten Island</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>jpsewerwater@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>718-619-0807</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Staten Island NY</t>
+        </is>
+      </c>
+      <c r="I134" t="n">
+        <v>100</v>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>drain cleaning service Staten Island NY</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 21:34 UTC (cycle 203)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L134"/>
+  <dimension ref="A1:L135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8238,6 +8238,58 @@
         </is>
       </c>
     </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Roof Replacement San Francisco</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>roofreplacementsanfrancisco.com</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>https://roofreplacementsanfrancisco.com/</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>info@roofreplacementsanfrancisco.com</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr"/>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>San Francisco CA</t>
+        </is>
+      </c>
+      <c r="I135" t="n">
+        <v>86</v>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>roof replacement San Francisco CA</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-28 21:36 UTC (cycle 204)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-28.xlsx
+++ b/output/leads_2026-09-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L135"/>
+  <dimension ref="A1:L136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8259,13 +8259,11 @@
           <t>https://roofreplacementsanfrancisco.com/</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr">
         <is>
           <t>info@roofreplacementsanfrancisco.com</t>
         </is>
       </c>
-      <c r="G135" t="inlineStr"/>
       <c r="H135" t="inlineStr">
         <is>
           <t>San Francisco CA</t>
@@ -8285,6 +8283,62 @@
         </is>
       </c>
       <c r="L135" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Ken's Plumbing, Aaron Sewer, &amp; Casper Heating</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>kensplumbingaaronsewer.com</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>https://kensplumbingaaronsewer.com/</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>kensplumbing1606@gmail.com</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>732-985-4428</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Edison NJ</t>
+        </is>
+      </c>
+      <c r="I136" t="n">
+        <v>90</v>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>plumbing company Edison NJ</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>

</xml_diff>